<commit_message>
derived: sync Wanfo component registry Excel
</commit_message>
<xml_diff>
--- a/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
+++ b/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
@@ -1589,7 +1589,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>直接实测</t>
+          <t>构件族直接实测｜SRC-ZG-WF-001 PDF p83 / 印刷p68 / 2.3.1.3 / 表2-40；样本与东/西缝逐件对应UNKNOWN</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1602,18 +1602,34 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>平均广395.5；厚280.5</t>
+          <t>实测组A 390×280；实测组B 401×281；均值广395.5；厚280.5</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>整殿实例长度由后续装配端点显式推导；Master reference length不得进入整殿实例</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="n">
+        <v>395.5</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>280.5</v>
+      </c>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>表2-40未将390×280与401×281逐一对应到东缝/西缝，禁止静默映射；报告归整为广26分、厚18分，仅作REPORT_INFERRED尺度分析，不作963历史设计值。图2-41示平梁与斗栱交接关系。</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>{"modeling_disposition":"DIRECT_MEASURED_SECTION / BUILDABLE","observed_section_samples_mm":[{"thickness":280,"width":390},{"thickness":281,"width":401}],"sample_to_instance_mapping":"UNKNOWN"}</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1643,7 +1659,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>直接实测</t>
+          <t>构件族直接实测｜SRC-ZG-WF-001 PDF p83 / 印刷p68 / 2.3.1.3 / 表2-40；样本与东/西缝逐件对应UNKNOWN</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1656,18 +1672,34 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>平均广395.5；厚280.5</t>
+          <t>实测组A 390×280；实测组B 401×281；均值广395.5；厚280.5</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>整殿实例长度由后续装配端点显式推导；Master reference length不得进入整殿实例</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
-      <c r="P21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="n">
+        <v>395.5</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>280.5</v>
+      </c>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="inlineStr"/>
-      <c r="T21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>表2-40未将390×280与401×281逐一对应到东缝/西缝，禁止静默映射；报告归整为广26分、厚18分，仅作REPORT_INFERRED尺度分析，不作963历史设计值。图2-41示平梁与斗栱交接关系。</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>{"modeling_disposition":"DIRECT_MEASURED_SECTION / BUILDABLE","observed_section_samples_mm":[{"thickness":280,"width":390},{"thickness":281,"width":401}],"sample_to_instance_mapping":"UNKNOWN"}</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1697,7 +1729,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>直接实测</t>
+          <t>数量/位置直接确认 + 山面型单一样本实测｜SRC-ZG-WF-001 PDF p83 / 印刷p68 / 2.3.1.3 / 表2-40；样本与东/西山逐件对应UNKNOWN</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1710,18 +1742,32 @@
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>广约346；厚未及</t>
+          <t>广346；厚未及（UNKNOWN）</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>整殿实例长度由后续装配端点显式推导；Master reference length不得进入整殿实例</t>
+        </is>
+      </c>
       <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="n">
+        <v>346</v>
+      </c>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>表2-40仅记录山面平梁广346mm，实测厚度未及/UNKNOWN；历史事实字段不得借用东西缝型280.5mm。为完整建模，另以同构件族东西缝实测均值截面比例显式补全 thickness=245.4mm，分类为PARAMETRIC_COMPLETION、可替换、非历史声明。报告将广归整为23分，仅作REPORT_INFERRED尺度分析。图2-41示平梁与斗栱交接关系。</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>{"modeling_disposition":"PARAMETRIC_COMPLETION / BUILDABLE / REPLACEABLE","observed_section_samples_mm":[{"thickness":null,"width":346}],"parametric_completion":{"classification":"PARAMETRIC_COMPLETION","field":"thickness_mm","formula":"346 * 280.5 / 395.5","historical_claim":false,"method":"preserve_east_west_seam_mean_section_aspect_ratio","note":"仅用于完整建模；不是报告实测厚度，也不是963年历史设计值。若后续取得山面平梁厚度直接证据，替换本值。","production_value_mm":245.4,"replaceable":true,"source_inputs_mm":{"east_west_mean_thickness_observed":280.5,"east_west_mean_width_observed":395.5,"gable_width_observed":346},"width_mm":{"classification":"PARAMETRIC_COMPLETION","historical_claim":false,"method":"generalize_single_observed_gable_sample_to_both_gable_instances","production_value_mm":346,"replaceable":true}},"sample_to_instance_mapping":"UNKNOWN"}</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1751,7 +1797,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>直接实测</t>
+          <t>数量/位置直接确认 + 山面型单一样本实测｜SRC-ZG-WF-001 PDF p83 / 印刷p68 / 2.3.1.3 / 表2-40；样本与东/西山逐件对应UNKNOWN</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1764,18 +1810,32 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>广约346；厚未及</t>
+          <t>广346；厚未及（UNKNOWN）</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>整殿实例长度由后续装配端点显式推导；Master reference length不得进入整殿实例</t>
+        </is>
+      </c>
       <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="n">
+        <v>346</v>
+      </c>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="inlineStr"/>
-      <c r="T23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>表2-40仅记录山面平梁广346mm，实测厚度未及/UNKNOWN；历史事实字段不得借用东西缝型280.5mm。为完整建模，另以同构件族东西缝实测均值截面比例显式补全 thickness=245.4mm，分类为PARAMETRIC_COMPLETION、可替换、非历史声明。报告将广归整为23分，仅作REPORT_INFERRED尺度分析。图2-41示平梁与斗栱交接关系。</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>{"modeling_disposition":"PARAMETRIC_COMPLETION / BUILDABLE / REPLACEABLE","observed_section_samples_mm":[{"thickness":null,"width":346}],"parametric_completion":{"classification":"PARAMETRIC_COMPLETION","field":"thickness_mm","formula":"346 * 280.5 / 395.5","historical_claim":false,"method":"preserve_east_west_seam_mean_section_aspect_ratio","note":"仅用于完整建模；不是报告实测厚度，也不是963年历史设计值。若后续取得山面平梁厚度直接证据，替换本值。","production_value_mm":245.4,"replaceable":true,"source_inputs_mm":{"east_west_mean_thickness_observed":280.5,"east_west_mean_width_observed":395.5,"gable_width_observed":346},"width_mm":{"classification":"PARAMETRIC_COMPLETION","historical_claim":false,"method":"generalize_single_observed_gable_sample_to_both_gable_instances","production_value_mm":346,"replaceable":true}},"sample_to_instance_mapping":"UNKNOWN"}</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -27847,7 +27907,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>02856c23e5ba34b9cb6bb07bb3e25afd69c87968</t>
+          <t>db2578b291547ed5816d095bdc543f2c51aede86</t>
         </is>
       </c>
     </row>
@@ -27859,7 +27919,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>e6299d8306fd4f58dac29a43230d387c2f63ca4056d002fd03803df02bb072a7</t>
+          <t>6709d7c9940368c51ac43b903e96ce442ed958f8b2385ed8825099a885f2dddf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T-036: rebase final approved state onto latest main
</commit_message>
<xml_diff>
--- a/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
+++ b/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.679</v>
+        <v>0.7140000000000001</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -2017,12 +2017,16 @@
           <t>需新建Master</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr"/>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="E71" s="3" t="n">
         <v>12</v>
       </c>
@@ -15618,10 +15622,14 @@
       </c>
       <c r="G203" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H203" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I203" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -15679,10 +15687,14 @@
       </c>
       <c r="G204" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H204" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I204" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -15740,10 +15752,14 @@
       </c>
       <c r="G205" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H205" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I205" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -15801,10 +15817,14 @@
       </c>
       <c r="G206" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H206" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H206" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I206" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -15862,10 +15882,14 @@
       </c>
       <c r="G207" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H207" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I207" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -15923,10 +15947,14 @@
       </c>
       <c r="G208" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H208" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I208" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -15984,10 +16012,14 @@
       </c>
       <c r="G209" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H209" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I209" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -16045,10 +16077,14 @@
       </c>
       <c r="G210" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H210" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I210" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -16106,10 +16142,14 @@
       </c>
       <c r="G211" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H211" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I211" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -16167,10 +16207,14 @@
       </c>
       <c r="G212" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H212" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I212" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -16228,10 +16272,14 @@
       </c>
       <c r="G213" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H213" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I213" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -16289,10 +16337,14 @@
       </c>
       <c r="G214" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H214" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>CMP-DOU-BOTTOM-LONGKAI-001_MASTER</t>
+        </is>
+      </c>
       <c r="I214" s="3" t="inlineStr">
         <is>
           <t>报告直接称12组</t>
@@ -35996,7 +36048,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -36006,7 +36058,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -36017,7 +36069,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>67.9%</t>
+          <t>71.4%</t>
         </is>
       </c>
     </row>
@@ -36029,7 +36081,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>c526e8caea7aa96e70b68e6fdadc3ba2d6895ee5</t>
+          <t>d122aff5db6d6fc43cdf9017533f03981c374182</t>
         </is>
       </c>
     </row>
@@ -36041,7 +36093,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>6d5798777a85bd1b2c90b3b02999f0f9803e5f4c58c7f05793b2bbc8d63f7681</t>
+          <t>1aefcdcfed83447da79b1265ade15970a4b30d7005b027a78992a644aff35b2e</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T-040: final reconcile onto latest main before Ready+Merge
</commit_message>
<xml_diff>
--- a/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
+++ b/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.821</v>
+        <v>0.857</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>275</v>
+        <v>331</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -1070,12 +1070,16 @@
           <t>需新建Master</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="n">
         <v>56</v>
       </c>
@@ -16422,10 +16426,14 @@
       </c>
       <c r="G215" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H215" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I215" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16448,7 +16456,11 @@
       </c>
       <c r="U215" s="3" t="inlineStr"/>
       <c r="V215" s="3" t="inlineStr"/>
-      <c r="W215" s="3" t="inlineStr"/>
+      <c r="W215" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="3" t="inlineStr">
@@ -16483,10 +16495,14 @@
       </c>
       <c r="G216" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H216" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I216" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16509,7 +16525,11 @@
       </c>
       <c r="U216" s="3" t="inlineStr"/>
       <c r="V216" s="3" t="inlineStr"/>
-      <c r="W216" s="3" t="inlineStr"/>
+      <c r="W216" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
@@ -16544,10 +16564,14 @@
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H217" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I217" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16570,7 +16594,11 @@
       </c>
       <c r="U217" s="3" t="inlineStr"/>
       <c r="V217" s="3" t="inlineStr"/>
-      <c r="W217" s="3" t="inlineStr"/>
+      <c r="W217" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="3" t="inlineStr">
@@ -16605,10 +16633,14 @@
       </c>
       <c r="G218" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H218" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I218" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16631,7 +16663,11 @@
       </c>
       <c r="U218" s="3" t="inlineStr"/>
       <c r="V218" s="3" t="inlineStr"/>
-      <c r="W218" s="3" t="inlineStr"/>
+      <c r="W218" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
@@ -16666,10 +16702,14 @@
       </c>
       <c r="G219" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H219" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I219" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16692,7 +16732,11 @@
       </c>
       <c r="U219" s="3" t="inlineStr"/>
       <c r="V219" s="3" t="inlineStr"/>
-      <c r="W219" s="3" t="inlineStr"/>
+      <c r="W219" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="3" t="inlineStr">
@@ -16727,10 +16771,14 @@
       </c>
       <c r="G220" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H220" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I220" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16753,7 +16801,11 @@
       </c>
       <c r="U220" s="3" t="inlineStr"/>
       <c r="V220" s="3" t="inlineStr"/>
-      <c r="W220" s="3" t="inlineStr"/>
+      <c r="W220" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
@@ -16788,10 +16840,14 @@
       </c>
       <c r="G221" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H221" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I221" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16814,7 +16870,11 @@
       </c>
       <c r="U221" s="3" t="inlineStr"/>
       <c r="V221" s="3" t="inlineStr"/>
-      <c r="W221" s="3" t="inlineStr"/>
+      <c r="W221" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="3" t="inlineStr">
@@ -16849,10 +16909,14 @@
       </c>
       <c r="G222" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H222" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I222" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16875,7 +16939,11 @@
       </c>
       <c r="U222" s="3" t="inlineStr"/>
       <c r="V222" s="3" t="inlineStr"/>
-      <c r="W222" s="3" t="inlineStr"/>
+      <c r="W222" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
@@ -16910,10 +16978,14 @@
       </c>
       <c r="G223" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H223" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I223" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16936,7 +17008,11 @@
       </c>
       <c r="U223" s="3" t="inlineStr"/>
       <c r="V223" s="3" t="inlineStr"/>
-      <c r="W223" s="3" t="inlineStr"/>
+      <c r="W223" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="3" t="inlineStr">
@@ -16971,10 +17047,14 @@
       </c>
       <c r="G224" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H224" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I224" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -16997,7 +17077,11 @@
       </c>
       <c r="U224" s="3" t="inlineStr"/>
       <c r="V224" s="3" t="inlineStr"/>
-      <c r="W224" s="3" t="inlineStr"/>
+      <c r="W224" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="3" t="inlineStr">
@@ -17032,10 +17116,14 @@
       </c>
       <c r="G225" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H225" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I225" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17058,7 +17146,11 @@
       </c>
       <c r="U225" s="3" t="inlineStr"/>
       <c r="V225" s="3" t="inlineStr"/>
-      <c r="W225" s="3" t="inlineStr"/>
+      <c r="W225" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="3" t="inlineStr">
@@ -17093,10 +17185,14 @@
       </c>
       <c r="G226" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H226" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I226" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17119,7 +17215,11 @@
       </c>
       <c r="U226" s="3" t="inlineStr"/>
       <c r="V226" s="3" t="inlineStr"/>
-      <c r="W226" s="3" t="inlineStr"/>
+      <c r="W226" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="3" t="inlineStr">
@@ -17154,10 +17254,14 @@
       </c>
       <c r="G227" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H227" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I227" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17180,7 +17284,11 @@
       </c>
       <c r="U227" s="3" t="inlineStr"/>
       <c r="V227" s="3" t="inlineStr"/>
-      <c r="W227" s="3" t="inlineStr"/>
+      <c r="W227" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="3" t="inlineStr">
@@ -17215,10 +17323,14 @@
       </c>
       <c r="G228" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H228" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I228" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17241,7 +17353,11 @@
       </c>
       <c r="U228" s="3" t="inlineStr"/>
       <c r="V228" s="3" t="inlineStr"/>
-      <c r="W228" s="3" t="inlineStr"/>
+      <c r="W228" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
@@ -17276,10 +17392,14 @@
       </c>
       <c r="G229" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H229" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I229" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17302,7 +17422,11 @@
       </c>
       <c r="U229" s="3" t="inlineStr"/>
       <c r="V229" s="3" t="inlineStr"/>
-      <c r="W229" s="3" t="inlineStr"/>
+      <c r="W229" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="3" t="inlineStr">
@@ -17337,10 +17461,14 @@
       </c>
       <c r="G230" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H230" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I230" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17363,7 +17491,11 @@
       </c>
       <c r="U230" s="3" t="inlineStr"/>
       <c r="V230" s="3" t="inlineStr"/>
-      <c r="W230" s="3" t="inlineStr"/>
+      <c r="W230" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="3" t="inlineStr">
@@ -17398,10 +17530,14 @@
       </c>
       <c r="G231" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H231" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I231" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17424,7 +17560,11 @@
       </c>
       <c r="U231" s="3" t="inlineStr"/>
       <c r="V231" s="3" t="inlineStr"/>
-      <c r="W231" s="3" t="inlineStr"/>
+      <c r="W231" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="3" t="inlineStr">
@@ -17459,10 +17599,14 @@
       </c>
       <c r="G232" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H232" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I232" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17485,7 +17629,11 @@
       </c>
       <c r="U232" s="3" t="inlineStr"/>
       <c r="V232" s="3" t="inlineStr"/>
-      <c r="W232" s="3" t="inlineStr"/>
+      <c r="W232" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="3" t="inlineStr">
@@ -17520,10 +17668,14 @@
       </c>
       <c r="G233" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H233" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I233" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17546,7 +17698,11 @@
       </c>
       <c r="U233" s="3" t="inlineStr"/>
       <c r="V233" s="3" t="inlineStr"/>
-      <c r="W233" s="3" t="inlineStr"/>
+      <c r="W233" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="3" t="inlineStr">
@@ -17581,10 +17737,14 @@
       </c>
       <c r="G234" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H234" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H234" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I234" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17607,7 +17767,11 @@
       </c>
       <c r="U234" s="3" t="inlineStr"/>
       <c r="V234" s="3" t="inlineStr"/>
-      <c r="W234" s="3" t="inlineStr"/>
+      <c r="W234" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="3" t="inlineStr">
@@ -17642,10 +17806,14 @@
       </c>
       <c r="G235" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H235" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I235" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17668,7 +17836,11 @@
       </c>
       <c r="U235" s="3" t="inlineStr"/>
       <c r="V235" s="3" t="inlineStr"/>
-      <c r="W235" s="3" t="inlineStr"/>
+      <c r="W235" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="3" t="inlineStr">
@@ -17703,10 +17875,14 @@
       </c>
       <c r="G236" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H236" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I236" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17729,7 +17905,11 @@
       </c>
       <c r="U236" s="3" t="inlineStr"/>
       <c r="V236" s="3" t="inlineStr"/>
-      <c r="W236" s="3" t="inlineStr"/>
+      <c r="W236" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
@@ -17764,10 +17944,14 @@
       </c>
       <c r="G237" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H237" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I237" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17790,7 +17974,11 @@
       </c>
       <c r="U237" s="3" t="inlineStr"/>
       <c r="V237" s="3" t="inlineStr"/>
-      <c r="W237" s="3" t="inlineStr"/>
+      <c r="W237" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="3" t="inlineStr">
@@ -17825,10 +18013,14 @@
       </c>
       <c r="G238" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H238" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H238" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I238" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17851,7 +18043,11 @@
       </c>
       <c r="U238" s="3" t="inlineStr"/>
       <c r="V238" s="3" t="inlineStr"/>
-      <c r="W238" s="3" t="inlineStr"/>
+      <c r="W238" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="3" t="inlineStr">
@@ -17886,10 +18082,14 @@
       </c>
       <c r="G239" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H239" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I239" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17912,7 +18112,11 @@
       </c>
       <c r="U239" s="3" t="inlineStr"/>
       <c r="V239" s="3" t="inlineStr"/>
-      <c r="W239" s="3" t="inlineStr"/>
+      <c r="W239" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="3" t="inlineStr">
@@ -17947,10 +18151,14 @@
       </c>
       <c r="G240" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H240" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H240" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I240" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -17973,7 +18181,11 @@
       </c>
       <c r="U240" s="3" t="inlineStr"/>
       <c r="V240" s="3" t="inlineStr"/>
-      <c r="W240" s="3" t="inlineStr"/>
+      <c r="W240" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
@@ -18008,10 +18220,14 @@
       </c>
       <c r="G241" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H241" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H241" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I241" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18034,7 +18250,11 @@
       </c>
       <c r="U241" s="3" t="inlineStr"/>
       <c r="V241" s="3" t="inlineStr"/>
-      <c r="W241" s="3" t="inlineStr"/>
+      <c r="W241" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="3" t="inlineStr">
@@ -18069,10 +18289,14 @@
       </c>
       <c r="G242" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H242" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H242" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I242" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18095,7 +18319,11 @@
       </c>
       <c r="U242" s="3" t="inlineStr"/>
       <c r="V242" s="3" t="inlineStr"/>
-      <c r="W242" s="3" t="inlineStr"/>
+      <c r="W242" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
@@ -18130,10 +18358,14 @@
       </c>
       <c r="G243" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H243" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H243" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I243" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18156,7 +18388,11 @@
       </c>
       <c r="U243" s="3" t="inlineStr"/>
       <c r="V243" s="3" t="inlineStr"/>
-      <c r="W243" s="3" t="inlineStr"/>
+      <c r="W243" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="3" t="inlineStr">
@@ -18191,10 +18427,14 @@
       </c>
       <c r="G244" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H244" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H244" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I244" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18217,7 +18457,11 @@
       </c>
       <c r="U244" s="3" t="inlineStr"/>
       <c r="V244" s="3" t="inlineStr"/>
-      <c r="W244" s="3" t="inlineStr"/>
+      <c r="W244" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="3" t="inlineStr">
@@ -18252,10 +18496,14 @@
       </c>
       <c r="G245" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H245" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H245" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I245" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18278,7 +18526,11 @@
       </c>
       <c r="U245" s="3" t="inlineStr"/>
       <c r="V245" s="3" t="inlineStr"/>
-      <c r="W245" s="3" t="inlineStr"/>
+      <c r="W245" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="3" t="inlineStr">
@@ -18313,10 +18565,14 @@
       </c>
       <c r="G246" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H246" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H246" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I246" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18339,7 +18595,11 @@
       </c>
       <c r="U246" s="3" t="inlineStr"/>
       <c r="V246" s="3" t="inlineStr"/>
-      <c r="W246" s="3" t="inlineStr"/>
+      <c r="W246" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
@@ -18374,10 +18634,14 @@
       </c>
       <c r="G247" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H247" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H247" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I247" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18400,7 +18664,11 @@
       </c>
       <c r="U247" s="3" t="inlineStr"/>
       <c r="V247" s="3" t="inlineStr"/>
-      <c r="W247" s="3" t="inlineStr"/>
+      <c r="W247" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="3" t="inlineStr">
@@ -18435,10 +18703,14 @@
       </c>
       <c r="G248" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H248" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H248" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I248" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18461,7 +18733,11 @@
       </c>
       <c r="U248" s="3" t="inlineStr"/>
       <c r="V248" s="3" t="inlineStr"/>
-      <c r="W248" s="3" t="inlineStr"/>
+      <c r="W248" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="3" t="inlineStr">
@@ -18496,10 +18772,14 @@
       </c>
       <c r="G249" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H249" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H249" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I249" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18522,7 +18802,11 @@
       </c>
       <c r="U249" s="3" t="inlineStr"/>
       <c r="V249" s="3" t="inlineStr"/>
-      <c r="W249" s="3" t="inlineStr"/>
+      <c r="W249" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="3" t="inlineStr">
@@ -18557,10 +18841,14 @@
       </c>
       <c r="G250" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H250" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H250" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I250" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18583,7 +18871,11 @@
       </c>
       <c r="U250" s="3" t="inlineStr"/>
       <c r="V250" s="3" t="inlineStr"/>
-      <c r="W250" s="3" t="inlineStr"/>
+      <c r="W250" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="3" t="inlineStr">
@@ -18618,10 +18910,14 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H251" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H251" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I251" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18644,7 +18940,11 @@
       </c>
       <c r="U251" s="3" t="inlineStr"/>
       <c r="V251" s="3" t="inlineStr"/>
-      <c r="W251" s="3" t="inlineStr"/>
+      <c r="W251" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="3" t="inlineStr">
@@ -18679,10 +18979,14 @@
       </c>
       <c r="G252" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H252" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H252" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I252" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18705,7 +19009,11 @@
       </c>
       <c r="U252" s="3" t="inlineStr"/>
       <c r="V252" s="3" t="inlineStr"/>
-      <c r="W252" s="3" t="inlineStr"/>
+      <c r="W252" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="3" t="inlineStr">
@@ -18740,10 +19048,14 @@
       </c>
       <c r="G253" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H253" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H253" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I253" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18766,7 +19078,11 @@
       </c>
       <c r="U253" s="3" t="inlineStr"/>
       <c r="V253" s="3" t="inlineStr"/>
-      <c r="W253" s="3" t="inlineStr"/>
+      <c r="W253" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="3" t="inlineStr">
@@ -18801,10 +19117,14 @@
       </c>
       <c r="G254" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H254" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H254" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I254" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18827,7 +19147,11 @@
       </c>
       <c r="U254" s="3" t="inlineStr"/>
       <c r="V254" s="3" t="inlineStr"/>
-      <c r="W254" s="3" t="inlineStr"/>
+      <c r="W254" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="3" t="inlineStr">
@@ -18862,10 +19186,14 @@
       </c>
       <c r="G255" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H255" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H255" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I255" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18888,7 +19216,11 @@
       </c>
       <c r="U255" s="3" t="inlineStr"/>
       <c r="V255" s="3" t="inlineStr"/>
-      <c r="W255" s="3" t="inlineStr"/>
+      <c r="W255" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="3" t="inlineStr">
@@ -18923,10 +19255,14 @@
       </c>
       <c r="G256" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H256" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H256" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I256" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -18949,7 +19285,11 @@
       </c>
       <c r="U256" s="3" t="inlineStr"/>
       <c r="V256" s="3" t="inlineStr"/>
-      <c r="W256" s="3" t="inlineStr"/>
+      <c r="W256" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="3" t="inlineStr">
@@ -18984,10 +19324,14 @@
       </c>
       <c r="G257" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H257" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H257" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I257" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19010,7 +19354,11 @@
       </c>
       <c r="U257" s="3" t="inlineStr"/>
       <c r="V257" s="3" t="inlineStr"/>
-      <c r="W257" s="3" t="inlineStr"/>
+      <c r="W257" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="3" t="inlineStr">
@@ -19045,10 +19393,14 @@
       </c>
       <c r="G258" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H258" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H258" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I258" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19071,7 +19423,11 @@
       </c>
       <c r="U258" s="3" t="inlineStr"/>
       <c r="V258" s="3" t="inlineStr"/>
-      <c r="W258" s="3" t="inlineStr"/>
+      <c r="W258" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="inlineStr">
@@ -19106,10 +19462,14 @@
       </c>
       <c r="G259" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H259" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H259" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I259" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19132,7 +19492,11 @@
       </c>
       <c r="U259" s="3" t="inlineStr"/>
       <c r="V259" s="3" t="inlineStr"/>
-      <c r="W259" s="3" t="inlineStr"/>
+      <c r="W259" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="3" t="inlineStr">
@@ -19167,10 +19531,14 @@
       </c>
       <c r="G260" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H260" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H260" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I260" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19193,7 +19561,11 @@
       </c>
       <c r="U260" s="3" t="inlineStr"/>
       <c r="V260" s="3" t="inlineStr"/>
-      <c r="W260" s="3" t="inlineStr"/>
+      <c r="W260" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="3" t="inlineStr">
@@ -19228,10 +19600,14 @@
       </c>
       <c r="G261" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H261" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I261" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19254,7 +19630,11 @@
       </c>
       <c r="U261" s="3" t="inlineStr"/>
       <c r="V261" s="3" t="inlineStr"/>
-      <c r="W261" s="3" t="inlineStr"/>
+      <c r="W261" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="3" t="inlineStr">
@@ -19289,10 +19669,14 @@
       </c>
       <c r="G262" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H262" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H262" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I262" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19315,7 +19699,11 @@
       </c>
       <c r="U262" s="3" t="inlineStr"/>
       <c r="V262" s="3" t="inlineStr"/>
-      <c r="W262" s="3" t="inlineStr"/>
+      <c r="W262" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="3" t="inlineStr">
@@ -19350,10 +19738,14 @@
       </c>
       <c r="G263" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H263" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H263" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I263" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19376,7 +19768,11 @@
       </c>
       <c r="U263" s="3" t="inlineStr"/>
       <c r="V263" s="3" t="inlineStr"/>
-      <c r="W263" s="3" t="inlineStr"/>
+      <c r="W263" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="3" t="inlineStr">
@@ -19411,10 +19807,14 @@
       </c>
       <c r="G264" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H264" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H264" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I264" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19437,7 +19837,11 @@
       </c>
       <c r="U264" s="3" t="inlineStr"/>
       <c r="V264" s="3" t="inlineStr"/>
-      <c r="W264" s="3" t="inlineStr"/>
+      <c r="W264" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="inlineStr">
@@ -19472,10 +19876,14 @@
       </c>
       <c r="G265" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H265" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H265" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I265" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19498,7 +19906,11 @@
       </c>
       <c r="U265" s="3" t="inlineStr"/>
       <c r="V265" s="3" t="inlineStr"/>
-      <c r="W265" s="3" t="inlineStr"/>
+      <c r="W265" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="3" t="inlineStr">
@@ -19533,10 +19945,14 @@
       </c>
       <c r="G266" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H266" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H266" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I266" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19559,7 +19975,11 @@
       </c>
       <c r="U266" s="3" t="inlineStr"/>
       <c r="V266" s="3" t="inlineStr"/>
-      <c r="W266" s="3" t="inlineStr"/>
+      <c r="W266" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
@@ -19594,10 +20014,14 @@
       </c>
       <c r="G267" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H267" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H267" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I267" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19620,7 +20044,11 @@
       </c>
       <c r="U267" s="3" t="inlineStr"/>
       <c r="V267" s="3" t="inlineStr"/>
-      <c r="W267" s="3" t="inlineStr"/>
+      <c r="W267" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="3" t="inlineStr">
@@ -19655,10 +20083,14 @@
       </c>
       <c r="G268" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H268" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H268" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I268" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19681,7 +20113,11 @@
       </c>
       <c r="U268" s="3" t="inlineStr"/>
       <c r="V268" s="3" t="inlineStr"/>
-      <c r="W268" s="3" t="inlineStr"/>
+      <c r="W268" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="3" t="inlineStr">
@@ -19716,10 +20152,14 @@
       </c>
       <c r="G269" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H269" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H269" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I269" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19742,7 +20182,11 @@
       </c>
       <c r="U269" s="3" t="inlineStr"/>
       <c r="V269" s="3" t="inlineStr"/>
-      <c r="W269" s="3" t="inlineStr"/>
+      <c r="W269" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_1_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="3" t="inlineStr">
@@ -19777,10 +20221,14 @@
       </c>
       <c r="G270" s="3" t="inlineStr">
         <is>
-          <t>MASTER_REQUIRED_PENDING</t>
-        </is>
-      </c>
-      <c r="H270" s="3" t="inlineStr"/>
+          <t>APPROVED_MASTER_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="H270" s="3" t="inlineStr">
+        <is>
+          <t>CMP-GONG-HUAGONG-001_MASTER</t>
+        </is>
+      </c>
       <c r="I270" s="3" t="inlineStr">
         <is>
           <t>每方向单元一、二跳各1</t>
@@ -19803,7 +20251,11 @@
       </c>
       <c r="U270" s="3" t="inlineStr"/>
       <c r="V270" s="3" t="inlineStr"/>
-      <c r="W270" s="3" t="inlineStr"/>
+      <c r="W270" s="3" t="inlineStr">
+        <is>
+          <t>{"historical_standalone_full_length_status":"UNRESOLVED","master_variant":"JUMP_2_HUAGONG","reference_specimen_length_applies_to_instance":false}</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="3" t="inlineStr">
@@ -36532,7 +36984,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
@@ -36542,7 +36994,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -36553,7 +37005,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>82.1%</t>
+          <t>85.7%</t>
         </is>
       </c>
     </row>
@@ -36565,7 +37017,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>47d945e6fa5dc495d569b88a46f7a61a57539e80</t>
+          <t>0e0c084f42deffc068b8a8bae25bac596a74cef2</t>
         </is>
       </c>
     </row>
@@ -36577,7 +37029,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>c10083efe039f378967b13a9b84944c6dcc336dc02a7ccc9acf4379966acf8d3</t>
+          <t>cc43517f53601ace183bcb05d09f64c5ddad8fa3134d6838b379880b29001c37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
D-263: sync reconciled Stage1 derived views
</commit_message>
<xml_diff>
--- a/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
+++ b/docs/evidence/zhenguo_wanfo/derived/P3_WANFO_COMPONENT_INSTANCE_REGISTRY_CURRENT.xlsx
@@ -627,15 +627,15 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>已批准 Master</t>
+          <t>已覆盖 Master-scope 类型</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>PRODUCT_OWNER_APPROVED Master available</t>
+          <t>Master-scope对象类型中已有APPROVED_MASTER_AVAILABLE绑定的类型数</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -647,15 +647,15 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>待完成 Master</t>
+          <t>待完成 Master-scope 类型</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Master范围 - 已批准Master</t>
+          <t>Master-scope对象类型中尚未覆盖的类型数</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -667,15 +667,15 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Master完成度</t>
+          <t>Master-scope 覆盖率</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.893</v>
+        <v>1</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>已批准Master / Stage1 Master范围</t>
+          <t>已覆盖Master-scope对象类型 / Stage1 Master范围；不得用Master family数量作分子</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -687,38 +687,58 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>已绑定Master的登记记录</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>363</v>
+          <t>已批准 Master families</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>25</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>仅表示V008登记行覆盖数，不等于物理构件总件数</t>
+          <t>PRODUCT_OWNER_APPROVED Master family数量；与object type覆盖数是不同维度</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>COMPLETE</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>已绑定Master的登记记录</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>363</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>仅表示V008登记行覆盖数，不等于物理构件总件数</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>PENDING_SOURCE_BINDING</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>仍在V008之外、不得静默视为已覆盖的对象</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -37132,7 +37152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -37244,114 +37264,124 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>已批准Master</t>
+          <t>已覆盖Master-scope类型</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>待完成Master</t>
+          <t>待完成Master-scope类型</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Master完成度</t>
+          <t>Master-scope覆盖率</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>89.3%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>源 GitHub 提交</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>b6b679b84f78a06e0d115f613f0f2d9fef30b271</t>
-        </is>
+          <t>已批准Master families</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>源 JSON SHA-256</t>
+          <t>源 GitHub 提交</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>c431aeaa54c665b0388a89f29a20e3255efc5877c8b6198baa3cc20da8365cbc</t>
+          <t>823c21f87610823bbfee734963fbaae31d4d714f</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>生成器版本</t>
+          <t>源 JSON SHA-256</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>1.0.2</t>
+          <t>4f32e65e5310ae4d92e7d20db5e8aa0fc0fa0b6923491827dfe94018dc242e97</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>生成器 SHA-256</t>
+          <t>生成器版本</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>e2695a9584e8a2c7e05f36713d92f5302595b5a877fd0b93f8615cfd4f35ab68</t>
+          <t>1.0.3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>同步规则</t>
+          <t>生成器 SHA-256</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>JSON先更新；Excel由自动流程生成。禁止人工修改Excel作为事实更新。</t>
+          <t>14f5092df95acb01ee1036ee5486fe791c78a5dbff93afa38ef3cc88cddb6383</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>版本规则</t>
+          <t>同步规则</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>CURRENT.xlsx对应CURRENT.json；Vxxx.xlsx对应同版本Vxxx.json快照。</t>
+          <t>JSON先更新；Excel由自动流程生成。禁止人工修改Excel作为事实更新。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>版本规则</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>CURRENT.xlsx对应CURRENT.json；Vxxx.xlsx对应同版本Vxxx.json快照。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>失败规则</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>自动生成失败时保持旧Excel并标记同步失败；不得假装已同步。</t>
         </is>

</xml_diff>